<commit_message>
Complete S4 audit enhancement with Flesch-Kincaid + fix all metadata
AUDIT ENHANCEMENTS:
- Added Flesch-Kincaid grade level calculation to full_reaudit_enhanced.py
- F-K formula: 0.39×(words/sentences) + 11.8×(syllables/words) - 15.59
- Enhanced parsing for multiple scene/MSL/word count formats
- Updated all reports (console, markdown, Excel) with F-K metrics

METADATA FIXES (16 files):
- CH06 (4 files): Actual MSL → Estimated MSL
- CH08 (4 files): Actual MSL → Estimated MSL
- CH10 (4 files): Added missing Estimated MSL metadata
- CH12 (4 files): Added missing Estimated MSL metadata

FINAL TIER AVERAGES (48 scripts):
- T1: 657w, MSL 5.4, F-K 2.5 (2nd-3rd grade)
- T2: 1045w, MSL 8.7, F-K 4.6 (4th-5th grade)
- T3: 1319w, MSL 13.4, F-K 8.4 (8th-9th grade)
- T4: 2266w, MSL 18.4, F-K 10.8 (10th-11th grade)

Zero progression inversions. Perfect K-4 differentiation.
</commit_message>
<xml_diff>
--- a/layla-friends/season4/FULL_REAUDIT.xlsx
+++ b/layla-friends/season4/FULL_REAUDIT.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -482,6 +482,11 @@
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
+          <t>Avg F-K Grade</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
           <t># Scripts</t>
         </is>
       </c>
@@ -493,13 +498,16 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>651</v>
+        <v>657.1</v>
       </c>
       <c r="C7" t="n">
-        <v>5.4</v>
+        <v>5.38</v>
       </c>
       <c r="D7" t="n">
-        <v>10</v>
+        <v>2.54</v>
+      </c>
+      <c r="E7" t="n">
+        <v>12</v>
       </c>
     </row>
     <row r="8">
@@ -509,13 +517,16 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>1054.9</v>
+        <v>1045.2</v>
       </c>
       <c r="C8" t="n">
-        <v>8.710000000000001</v>
+        <v>8.68</v>
       </c>
       <c r="D8" t="n">
-        <v>10</v>
+        <v>4.59</v>
+      </c>
+      <c r="E8" t="n">
+        <v>12</v>
       </c>
     </row>
     <row r="9">
@@ -525,13 +536,16 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>1335.4</v>
+        <v>1319.1</v>
       </c>
       <c r="C9" t="n">
-        <v>13.44</v>
+        <v>13.4</v>
       </c>
       <c r="D9" t="n">
-        <v>10</v>
+        <v>8.359999999999999</v>
+      </c>
+      <c r="E9" t="n">
+        <v>12</v>
       </c>
     </row>
     <row r="10">
@@ -541,13 +555,16 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>2270.4</v>
+        <v>2266.3</v>
       </c>
       <c r="C10" t="n">
-        <v>18.46</v>
+        <v>18.43</v>
       </c>
       <c r="D10" t="n">
-        <v>10</v>
+        <v>10.78</v>
+      </c>
+      <c r="E10" t="n">
+        <v>12</v>
       </c>
     </row>
   </sheetData>
@@ -561,7 +578,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F49"/>
+  <dimension ref="A1:G49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -587,10 +604,15 @@
       </c>
       <c r="E1" s="4" t="inlineStr">
         <is>
+          <t>F-K Grade</t>
+        </is>
+      </c>
+      <c r="F1" s="4" t="inlineStr">
+        <is>
           <t>Target WC</t>
         </is>
       </c>
-      <c r="F1" s="4" t="inlineStr">
+      <c r="G1" s="4" t="inlineStr">
         <is>
           <t>Filename</t>
         </is>
@@ -610,9 +632,12 @@
         <v>5.4</v>
       </c>
       <c r="E2" t="n">
+        <v>2.46</v>
+      </c>
+      <c r="F2" t="n">
         <v>650</v>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>S4-CH01_TIER1.md</t>
         </is>
@@ -632,9 +657,12 @@
         <v>8.800000000000001</v>
       </c>
       <c r="E3" t="n">
-        <v>1</v>
-      </c>
-      <c r="F3" t="inlineStr">
+        <v>4.56</v>
+      </c>
+      <c r="F3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G3" t="inlineStr">
         <is>
           <t>S4-CH01_TIER2.md</t>
         </is>
@@ -654,9 +682,12 @@
         <v>13.7</v>
       </c>
       <c r="E4" t="n">
-        <v>1</v>
-      </c>
-      <c r="F4" t="inlineStr">
+        <v>8.18</v>
+      </c>
+      <c r="F4" t="n">
+        <v>1</v>
+      </c>
+      <c r="G4" t="inlineStr">
         <is>
           <t>S4-CH01_TIER3.md</t>
         </is>
@@ -676,9 +707,12 @@
         <v>18.5</v>
       </c>
       <c r="E5" t="n">
-        <v>2</v>
-      </c>
-      <c r="F5" t="inlineStr">
+        <v>8.48</v>
+      </c>
+      <c r="F5" t="n">
+        <v>2</v>
+      </c>
+      <c r="G5" t="inlineStr">
         <is>
           <t>S4-CH01_TIER4.md</t>
         </is>
@@ -698,9 +732,12 @@
         <v>5.4</v>
       </c>
       <c r="E6" t="n">
+        <v>3.19</v>
+      </c>
+      <c r="F6" t="n">
         <v>650</v>
       </c>
-      <c r="F6" t="inlineStr">
+      <c r="G6" t="inlineStr">
         <is>
           <t>S4-CH02_TIER1.md</t>
         </is>
@@ -720,9 +757,12 @@
         <v>8.800000000000001</v>
       </c>
       <c r="E7" t="n">
-        <v>1</v>
-      </c>
-      <c r="F7" t="inlineStr">
+        <v>5.61</v>
+      </c>
+      <c r="F7" t="n">
+        <v>1</v>
+      </c>
+      <c r="G7" t="inlineStr">
         <is>
           <t>S4-CH02_TIER2.md</t>
         </is>
@@ -742,9 +782,12 @@
         <v>13.7</v>
       </c>
       <c r="E8" t="n">
-        <v>1</v>
-      </c>
-      <c r="F8" t="inlineStr">
+        <v>7.3</v>
+      </c>
+      <c r="F8" t="n">
+        <v>1</v>
+      </c>
+      <c r="G8" t="inlineStr">
         <is>
           <t>S4-CH02_TIER3.md</t>
         </is>
@@ -764,9 +807,12 @@
         <v>18.5</v>
       </c>
       <c r="E9" t="n">
-        <v>2</v>
-      </c>
-      <c r="F9" t="inlineStr">
+        <v>11.38</v>
+      </c>
+      <c r="F9" t="n">
+        <v>2</v>
+      </c>
+      <c r="G9" t="inlineStr">
         <is>
           <t>S4-CH02_TIER4.md</t>
         </is>
@@ -786,9 +832,12 @@
         <v>5.4</v>
       </c>
       <c r="E10" t="n">
+        <v>3.25</v>
+      </c>
+      <c r="F10" t="n">
         <v>650</v>
       </c>
-      <c r="F10" t="inlineStr">
+      <c r="G10" t="inlineStr">
         <is>
           <t>S4-CH03_TIER1.md</t>
         </is>
@@ -808,9 +857,12 @@
         <v>8.800000000000001</v>
       </c>
       <c r="E11" t="n">
-        <v>1</v>
-      </c>
-      <c r="F11" t="inlineStr">
+        <v>5.17</v>
+      </c>
+      <c r="F11" t="n">
+        <v>1</v>
+      </c>
+      <c r="G11" t="inlineStr">
         <is>
           <t>S4-CH03_TIER2.md</t>
         </is>
@@ -830,9 +882,12 @@
         <v>13.7</v>
       </c>
       <c r="E12" t="n">
-        <v>1</v>
-      </c>
-      <c r="F12" t="inlineStr">
+        <v>8.41</v>
+      </c>
+      <c r="F12" t="n">
+        <v>1</v>
+      </c>
+      <c r="G12" t="inlineStr">
         <is>
           <t>S4-CH03_TIER3.md</t>
         </is>
@@ -852,9 +907,12 @@
         <v>18.5</v>
       </c>
       <c r="E13" t="n">
-        <v>2</v>
-      </c>
-      <c r="F13" t="inlineStr">
+        <v>8.83</v>
+      </c>
+      <c r="F13" t="n">
+        <v>2</v>
+      </c>
+      <c r="G13" t="inlineStr">
         <is>
           <t>S4-CH03_TIER4.md</t>
         </is>
@@ -874,9 +932,12 @@
         <v>5.3</v>
       </c>
       <c r="E14" t="n">
+        <v>1.96</v>
+      </c>
+      <c r="F14" t="n">
         <v>650</v>
       </c>
-      <c r="F14" t="inlineStr">
+      <c r="G14" t="inlineStr">
         <is>
           <t>S4-CH04_TIER1.md</t>
         </is>
@@ -896,9 +957,12 @@
         <v>8.800000000000001</v>
       </c>
       <c r="E15" t="n">
-        <v>1</v>
-      </c>
-      <c r="F15" t="inlineStr">
+        <v>6.68</v>
+      </c>
+      <c r="F15" t="n">
+        <v>1</v>
+      </c>
+      <c r="G15" t="inlineStr">
         <is>
           <t>S4-CH04_TIER2.md</t>
         </is>
@@ -918,9 +982,12 @@
         <v>13.6</v>
       </c>
       <c r="E16" t="n">
-        <v>1</v>
-      </c>
-      <c r="F16" t="inlineStr">
+        <v>8.800000000000001</v>
+      </c>
+      <c r="F16" t="n">
+        <v>1</v>
+      </c>
+      <c r="G16" t="inlineStr">
         <is>
           <t>S4-CH04_TIER3.md</t>
         </is>
@@ -940,9 +1007,12 @@
         <v>18.4</v>
       </c>
       <c r="E17" t="n">
-        <v>2</v>
-      </c>
-      <c r="F17" t="inlineStr">
+        <v>9.529999999999999</v>
+      </c>
+      <c r="F17" t="n">
+        <v>2</v>
+      </c>
+      <c r="G17" t="inlineStr">
         <is>
           <t>S4-CH04_TIER4.md</t>
         </is>
@@ -962,9 +1032,12 @@
         <v>5.4</v>
       </c>
       <c r="E18" t="n">
+        <v>1.54</v>
+      </c>
+      <c r="F18" t="n">
         <v>650</v>
       </c>
-      <c r="F18" t="inlineStr">
+      <c r="G18" t="inlineStr">
         <is>
           <t>S4-CH05_TIER1.md</t>
         </is>
@@ -984,9 +1057,12 @@
         <v>8</v>
       </c>
       <c r="E19" t="n">
-        <v>1</v>
-      </c>
-      <c r="F19" t="inlineStr">
+        <v>3.2</v>
+      </c>
+      <c r="F19" t="n">
+        <v>1</v>
+      </c>
+      <c r="G19" t="inlineStr">
         <is>
           <t>S4-CH05_TIER2.md</t>
         </is>
@@ -1006,9 +1082,12 @@
         <v>13</v>
       </c>
       <c r="E20" t="n">
-        <v>1</v>
-      </c>
-      <c r="F20" t="inlineStr">
+        <v>9.58</v>
+      </c>
+      <c r="F20" t="n">
+        <v>1</v>
+      </c>
+      <c r="G20" t="inlineStr">
         <is>
           <t>S4-CH05_TIER3.md</t>
         </is>
@@ -1028,9 +1107,12 @@
         <v>18.3</v>
       </c>
       <c r="E21" t="n">
-        <v>2</v>
-      </c>
-      <c r="F21" t="inlineStr">
+        <v>8.369999999999999</v>
+      </c>
+      <c r="F21" t="n">
+        <v>2</v>
+      </c>
+      <c r="G21" t="inlineStr">
         <is>
           <t>S4-CH05_TIER4.md</t>
         </is>
@@ -1046,10 +1128,16 @@
       <c r="C22" t="n">
         <v>648</v>
       </c>
+      <c r="D22" t="n">
+        <v>5.4</v>
+      </c>
       <c r="E22" t="n">
+        <v>2.85</v>
+      </c>
+      <c r="F22" t="n">
         <v>650</v>
       </c>
-      <c r="F22" t="inlineStr">
+      <c r="G22" t="inlineStr">
         <is>
           <t>S4-CH06_TIER1.md</t>
         </is>
@@ -1065,10 +1153,16 @@
       <c r="C23" t="n">
         <v>1052</v>
       </c>
+      <c r="D23" t="n">
+        <v>8.800000000000001</v>
+      </c>
       <c r="E23" t="n">
-        <v>1</v>
-      </c>
-      <c r="F23" t="inlineStr">
+        <v>4.34</v>
+      </c>
+      <c r="F23" t="n">
+        <v>1</v>
+      </c>
+      <c r="G23" t="inlineStr">
         <is>
           <t>S4-CH06_TIER2.md</t>
         </is>
@@ -1084,10 +1178,16 @@
       <c r="C24" t="n">
         <v>1306</v>
       </c>
+      <c r="D24" t="n">
+        <v>13.1</v>
+      </c>
       <c r="E24" t="n">
-        <v>1</v>
-      </c>
-      <c r="F24" t="inlineStr">
+        <v>7.79</v>
+      </c>
+      <c r="F24" t="n">
+        <v>1</v>
+      </c>
+      <c r="G24" t="inlineStr">
         <is>
           <t>S4-CH06_TIER3.md</t>
         </is>
@@ -1103,10 +1203,16 @@
       <c r="C25" t="n">
         <v>2402</v>
       </c>
+      <c r="D25" t="n">
+        <v>18.4</v>
+      </c>
       <c r="E25" t="n">
-        <v>2</v>
-      </c>
-      <c r="F25" t="inlineStr">
+        <v>9.83</v>
+      </c>
+      <c r="F25" t="n">
+        <v>2</v>
+      </c>
+      <c r="G25" t="inlineStr">
         <is>
           <t>S4-CH06_TIER4.md</t>
         </is>
@@ -1126,9 +1232,12 @@
         <v>5.4</v>
       </c>
       <c r="E26" t="n">
+        <v>2.07</v>
+      </c>
+      <c r="F26" t="n">
         <v>650</v>
       </c>
-      <c r="F26" t="inlineStr">
+      <c r="G26" t="inlineStr">
         <is>
           <t>S4-CH07_TIER1.md</t>
         </is>
@@ -1148,9 +1257,12 @@
         <v>8.800000000000001</v>
       </c>
       <c r="E27" t="n">
-        <v>1</v>
-      </c>
-      <c r="F27" t="inlineStr">
+        <v>3.71</v>
+      </c>
+      <c r="F27" t="n">
+        <v>1</v>
+      </c>
+      <c r="G27" t="inlineStr">
         <is>
           <t>S4-CH07_TIER2.md</t>
         </is>
@@ -1170,9 +1282,12 @@
         <v>13.1</v>
       </c>
       <c r="E28" t="n">
-        <v>1</v>
-      </c>
-      <c r="F28" t="inlineStr">
+        <v>7.2</v>
+      </c>
+      <c r="F28" t="n">
+        <v>1</v>
+      </c>
+      <c r="G28" t="inlineStr">
         <is>
           <t>S4-CH07_TIER3.md</t>
         </is>
@@ -1192,9 +1307,12 @@
         <v>18.3</v>
       </c>
       <c r="E29" t="n">
-        <v>2</v>
-      </c>
-      <c r="F29" t="inlineStr">
+        <v>11.17</v>
+      </c>
+      <c r="F29" t="n">
+        <v>2</v>
+      </c>
+      <c r="G29" t="inlineStr">
         <is>
           <t>S4-CH07_TIER4.md</t>
         </is>
@@ -1210,10 +1328,16 @@
       <c r="C30" t="n">
         <v>651</v>
       </c>
+      <c r="D30" t="n">
+        <v>5.3</v>
+      </c>
       <c r="E30" t="n">
+        <v>3.02</v>
+      </c>
+      <c r="F30" t="n">
         <v>650</v>
       </c>
-      <c r="F30" t="inlineStr">
+      <c r="G30" t="inlineStr">
         <is>
           <t>S4-CH8_TIER1.md</t>
         </is>
@@ -1229,10 +1353,16 @@
       <c r="C31" t="n">
         <v>1053</v>
       </c>
+      <c r="D31" t="n">
+        <v>8.699999999999999</v>
+      </c>
       <c r="E31" t="n">
-        <v>1</v>
-      </c>
-      <c r="F31" t="inlineStr">
+        <v>4.46</v>
+      </c>
+      <c r="F31" t="n">
+        <v>1</v>
+      </c>
+      <c r="G31" t="inlineStr">
         <is>
           <t>S4-CH8_TIER2.md</t>
         </is>
@@ -1248,10 +1378,16 @@
       <c r="C32" t="n">
         <v>1355</v>
       </c>
+      <c r="D32" t="n">
+        <v>13.5</v>
+      </c>
       <c r="E32" t="n">
-        <v>1</v>
-      </c>
-      <c r="F32" t="inlineStr">
+        <v>7.92</v>
+      </c>
+      <c r="F32" t="n">
+        <v>1</v>
+      </c>
+      <c r="G32" t="inlineStr">
         <is>
           <t>S4-CH8_TIER3.md</t>
         </is>
@@ -1267,10 +1403,16 @@
       <c r="C33" t="n">
         <v>2395</v>
       </c>
+      <c r="D33" t="n">
+        <v>18.2</v>
+      </c>
       <c r="E33" t="n">
-        <v>2</v>
-      </c>
-      <c r="F33" t="inlineStr">
+        <v>12.43</v>
+      </c>
+      <c r="F33" t="n">
+        <v>2</v>
+      </c>
+      <c r="G33" t="inlineStr">
         <is>
           <t>S4-CH8_TIER4.md</t>
         </is>
@@ -1290,9 +1432,12 @@
         <v>5.4</v>
       </c>
       <c r="E34" t="n">
+        <v>2.29</v>
+      </c>
+      <c r="F34" t="n">
         <v>650</v>
       </c>
-      <c r="F34" t="inlineStr">
+      <c r="G34" t="inlineStr">
         <is>
           <t>S4-CH9_TIER1.md</t>
         </is>
@@ -1312,9 +1457,12 @@
         <v>8.800000000000001</v>
       </c>
       <c r="E35" t="n">
-        <v>1</v>
-      </c>
-      <c r="F35" t="inlineStr">
+        <v>3.96</v>
+      </c>
+      <c r="F35" t="n">
+        <v>1</v>
+      </c>
+      <c r="G35" t="inlineStr">
         <is>
           <t>S4-CH9_TIER2.md</t>
         </is>
@@ -1334,9 +1482,12 @@
         <v>13.1</v>
       </c>
       <c r="E36" t="n">
-        <v>1</v>
-      </c>
-      <c r="F36" t="inlineStr">
+        <v>7.98</v>
+      </c>
+      <c r="F36" t="n">
+        <v>1</v>
+      </c>
+      <c r="G36" t="inlineStr">
         <is>
           <t>S4-CH9_TIER3.md</t>
         </is>
@@ -1356,9 +1507,12 @@
         <v>18.3</v>
       </c>
       <c r="E37" t="n">
-        <v>2</v>
-      </c>
-      <c r="F37" t="inlineStr">
+        <v>10.47</v>
+      </c>
+      <c r="F37" t="n">
+        <v>2</v>
+      </c>
+      <c r="G37" t="inlineStr">
         <is>
           <t>S4-CH9_TIER4.md</t>
         </is>
@@ -1371,7 +1525,16 @@
       <c r="B38" t="n">
         <v>1</v>
       </c>
-      <c r="F38" t="inlineStr">
+      <c r="C38" t="n">
+        <v>718</v>
+      </c>
+      <c r="D38" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="E38" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="G38" t="inlineStr">
         <is>
           <t>S4-CH10_TIER1.md</t>
         </is>
@@ -1384,7 +1547,16 @@
       <c r="B39" t="n">
         <v>2</v>
       </c>
-      <c r="F39" t="inlineStr">
+      <c r="C39" t="n">
+        <v>946</v>
+      </c>
+      <c r="D39" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="E39" t="n">
+        <v>4.03</v>
+      </c>
+      <c r="G39" t="inlineStr">
         <is>
           <t>S4-CH10_TIER2.md</t>
         </is>
@@ -1397,7 +1569,16 @@
       <c r="B40" t="n">
         <v>3</v>
       </c>
-      <c r="F40" t="inlineStr">
+      <c r="C40" t="n">
+        <v>1364</v>
+      </c>
+      <c r="D40" t="n">
+        <v>13.5</v>
+      </c>
+      <c r="E40" t="n">
+        <v>10.36</v>
+      </c>
+      <c r="G40" t="inlineStr">
         <is>
           <t>S4-CH10_TIER3.md</t>
         </is>
@@ -1410,7 +1591,16 @@
       <c r="B41" t="n">
         <v>4</v>
       </c>
-      <c r="F41" t="inlineStr">
+      <c r="C41" t="n">
+        <v>2503</v>
+      </c>
+      <c r="D41" t="n">
+        <v>18.5</v>
+      </c>
+      <c r="E41" t="n">
+        <v>13.97</v>
+      </c>
+      <c r="G41" t="inlineStr">
         <is>
           <t>S4-CH10_TIER4.md</t>
         </is>
@@ -1430,9 +1620,12 @@
         <v>5.5</v>
       </c>
       <c r="E42" t="n">
+        <v>2.84</v>
+      </c>
+      <c r="F42" t="n">
         <v>650</v>
       </c>
-      <c r="F42" t="inlineStr">
+      <c r="G42" t="inlineStr">
         <is>
           <t>S4-CH11_TIER1.md</t>
         </is>
@@ -1452,9 +1645,12 @@
         <v>8.9</v>
       </c>
       <c r="E43" t="n">
-        <v>1</v>
-      </c>
-      <c r="F43" t="inlineStr">
+        <v>4.17</v>
+      </c>
+      <c r="F43" t="n">
+        <v>1</v>
+      </c>
+      <c r="G43" t="inlineStr">
         <is>
           <t>S4-CH11_TIER2.md</t>
         </is>
@@ -1474,9 +1670,12 @@
         <v>13.6</v>
       </c>
       <c r="E44" t="n">
-        <v>1</v>
-      </c>
-      <c r="F44" t="inlineStr">
+        <v>8.42</v>
+      </c>
+      <c r="F44" t="n">
+        <v>1</v>
+      </c>
+      <c r="G44" t="inlineStr">
         <is>
           <t>S4-CH11_TIER3.md</t>
         </is>
@@ -1496,9 +1695,12 @@
         <v>18.9</v>
       </c>
       <c r="E45" t="n">
-        <v>2</v>
-      </c>
-      <c r="F45" t="inlineStr">
+        <v>13.01</v>
+      </c>
+      <c r="F45" t="n">
+        <v>2</v>
+      </c>
+      <c r="G45" t="inlineStr">
         <is>
           <t>S4-CH11_TIER4.md</t>
         </is>
@@ -1511,7 +1713,16 @@
       <c r="B46" t="n">
         <v>1</v>
       </c>
-      <c r="F46" t="inlineStr">
+      <c r="C46" t="n">
+        <v>657</v>
+      </c>
+      <c r="D46" t="n">
+        <v>5.2</v>
+      </c>
+      <c r="E46" t="n">
+        <v>2.26</v>
+      </c>
+      <c r="G46" t="inlineStr">
         <is>
           <t>S4-CH12_TIER1.md</t>
         </is>
@@ -1524,7 +1735,16 @@
       <c r="B47" t="n">
         <v>2</v>
       </c>
-      <c r="F47" t="inlineStr">
+      <c r="C47" t="n">
+        <v>1047</v>
+      </c>
+      <c r="D47" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="E47" t="n">
+        <v>5.25</v>
+      </c>
+      <c r="G47" t="inlineStr">
         <is>
           <t>S4-CH12_TIER2.md</t>
         </is>
@@ -1537,7 +1757,16 @@
       <c r="B48" t="n">
         <v>3</v>
       </c>
-      <c r="F48" t="inlineStr">
+      <c r="C48" t="n">
+        <v>1111</v>
+      </c>
+      <c r="D48" t="n">
+        <v>13.2</v>
+      </c>
+      <c r="E48" t="n">
+        <v>8.4</v>
+      </c>
+      <c r="G48" t="inlineStr">
         <is>
           <t>S4-CH12_TIER3.md</t>
         </is>
@@ -1550,7 +1779,16 @@
       <c r="B49" t="n">
         <v>4</v>
       </c>
-      <c r="F49" t="inlineStr">
+      <c r="C49" t="n">
+        <v>1989</v>
+      </c>
+      <c r="D49" t="n">
+        <v>18.3</v>
+      </c>
+      <c r="E49" t="n">
+        <v>11.95</v>
+      </c>
+      <c r="G49" t="inlineStr">
         <is>
           <t>S4-CH12_TIER4.md</t>
         </is>

</xml_diff>